<commit_message>
docs(cpq): document the LLM-first coverage follow-up in the implementation doc and xlsx
Companion to the test commit on this branch. Adds a "Follow-up" section
to CPQ_ASK_OFFTOPIC_INTENT_FALSE_POSITIVE_FIXES_2026-08-13.md and a new
"Followup-LLM-First-Coverage" sheet to the xlsx report, both covering:
issue (regex enumeration can't generalize + the great/perfect fix's own
new gap), root cause (no LLM fallback at the point these two detectors
are consulted), fix (found the LLM-first gateway already covers this,
added proof tests instead of duplicating it), the known guided_mode
gap this doesn't close, and the 3 independent-review findings that
were fixed before this commit.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/CPQ_OffTopic_Intent_Failed_Testcases_RootCause_Fix_2026-08-13.xlsx
+++ b/docs/CPQ_OffTopic_Intent_Failed_Testcases_RootCause_Fix_2026-08-13.xlsx
@@ -10,6 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10-OffTopic" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4-Intent" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Followup-LLM-First-Coverage" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -19,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -31,8 +32,11 @@
       <b val="1"/>
       <color rgb="00FFFFFF"/>
     </font>
+    <font>
+      <b val="1"/>
+    </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -57,6 +61,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FFF3CD"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00DDEBF7"/>
       </patternFill>
     </fill>
   </fills>
@@ -86,7 +95,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -99,6 +108,12 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -552,9 +567,6 @@
           <t>https://github.com/Giggso-Inc/aryx-enterprise/pull/new/fix/cpq-offtopic-approval-qa-false-positives</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr"/>
-      <c r="D4" t="inlineStr"/>
-      <c r="E4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -567,9 +579,6 @@
           <t>fix/cpq-offtopic-approval-qa-false-positives</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr"/>
-      <c r="D5" t="inlineStr"/>
-      <c r="E5" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -4498,4 +4507,130 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="110" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>Detail</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="6" t="inlineStr">
+        <is>
+          <t>PR / Branch</t>
+        </is>
+      </c>
+      <c r="B2" s="7" t="inlineStr">
+        <is>
+          <t>fix/cpq-approval-llm-first-coverage-proof (aryx-enterprise, base dev-rv)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="6" t="inlineStr">
+        <is>
+          <t>Question raised</t>
+        </is>
+      </c>
+      <c r="B3" s="7" t="inlineStr">
+        <is>
+          <t>Does the regex-only fix (previous PR) generalize to any phrasing, or does it only cover the exact reported test cases?</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="6" t="inlineStr">
+        <is>
+          <t>Issue</t>
+        </is>
+      </c>
+      <c r="B4" s="7" t="inlineStr">
+        <is>
+          <t>detect_approval/detect_qa_question (engine.py) are pure anchored regex with no semantic fallback. Regex is an enumeration -- it cannot cover every way a customer phrases approval ("sounds good to me", "works for me"). The D42 fix (narrowing great/perfect to a whole-message-only pattern) also introduced a new gap: "Perfect, let's go" no longer matches the regex either.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>Root Cause</t>
+        </is>
+      </c>
+      <c r="B5" s="7" t="inlineStr">
+        <is>
+          <t>No LLM-based fallback existed for these two detectors at the point they are consulted directly -- unlike other categories already migrated to intent_gateway.py's LLM-first classifier.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="6" t="inlineStr">
+        <is>
+          <t>Fix Implemented</t>
+        </is>
+      </c>
+      <c r="B6" s="7" t="inlineStr">
+        <is>
+          <t>Investigated adding a NEW LLM-fallback helper (the originally recommended approach) and found it unnecessary: APPROVAL and QA_QUESTION are ALREADY wired into _dispatch_intent_result (ask_api.py, commits 06d4c69 / b7151cc) as no-target, non-mutating categories -- classify_intent's quarantine (confidence=HIGH + evidence_span present) is the only gate, no dependency on the regex at all, and cpq_llm_first_enabled defaults to True. Added 3 tests proving this coverage instead of duplicating existing infrastructure: 2 in tests/test_cpq_intent_gateway.py (classify_intent resolves 'sounds good to me...' and 'Perfect, let's go' to APPROVAL/HIGH) and 1 integration test in tests/test_cpq_2026_07_28_fixes.py proving _dispatch_intent_result's APPROVAL branch submits the payload with detect_approval patched to return False.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="6" t="inlineStr">
+        <is>
+          <t>Known gap NOT closed</t>
+        </is>
+      </c>
+      <c r="B7" s="7" t="inlineStr">
+        <is>
+          <t>session.guided_mode=True skips the LLM-first gateway entirely (ask_api.py STEP-6 gate) -- guided-mode sessions still rely solely on the regex for approval detection.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="6" t="inlineStr">
+        <is>
+          <t>Independent review findings (all fixed)</t>
+        </is>
+      </c>
+      <c r="B8" s="7" t="inlineStr">
+        <is>
+          <t>HIGH: a test asserted engine.detect_approval.assert_not_called() as proof the LLM path skips the regex, but intent_gateway.py never calls that method for ANY category -- tautological, not evidence. Replaced with a real integration test at the correct call site. MEDIUM: the guided_mode gap was undocumented -- now documented. LOW: 2 new tests left engine.detect_change_* mocks unset, unlike file convention -- fixed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="6" t="inlineStr">
+        <is>
+          <t>Verification</t>
+        </is>
+      </c>
+      <c r="B9" s="7" t="inlineStr">
+        <is>
+          <t>tests/test_cpq_intent_gateway.py: 25 passed. tests/test_cpq_2026_07_28_fixes.py -k approval: 7 passed. (Full file has pre-existing, unrelated tests that hang in this sandbox due to a real network-access limitation, confirmed via bisection to predate and be unrelated to this change.)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
docs(cpq): correct D42 framing from 'gap' to 'fixed regression' per raven review
Companion to the regex fix commit on this branch. Updates D42's row in
the implementation doc and xlsx to describe the great/perfect
whole-message-only pattern's own regression (breaking "Great, let's
go" / "Perfect, that works") and how it was fixed, rather than leaving
the original text implying no further issue.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/CPQ_OffTopic_Intent_Failed_Testcases_RootCause_Fix_2026-08-13.xlsx
+++ b/docs/CPQ_OffTopic_Intent_Failed_Testcases_RootCause_Fix_2026-08-13.xlsx
@@ -552,9 +552,6 @@
           <t>https://github.com/Giggso-Inc/aryx-enterprise/pull/new/fix/cpq-offtopic-approval-qa-false-positives</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr"/>
-      <c r="D4" t="inlineStr"/>
-      <c r="E4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -567,9 +564,6 @@
           <t>fix/cpq-offtopic-approval-qa-false-positives</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr"/>
-      <c r="D5" t="inlineStr"/>
-      <c r="E5" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3320,7 +3314,7 @@
       </c>
       <c r="K44" s="4" t="inlineStr">
         <is>
-          <t>Moved great/perfect out of the general alternation into a standalone-reply-only pattern: ^(?:great|perfect)\s*[!.]*$ -- only matches when the entire trimmed message IS just that word (+ optional punctuation).</t>
+          <t>Moved great/perfect out of the general alternation into a standalone-reply-only pattern: ^(?:great|perfect)\s*[!.]*$ -- only matches when the entire trimmed message IS just that word (+ optional punctuation). UPDATE (raven review on PR #192): this whole-message-only pattern also broke previously-working combined phrasings ('Great, let's go', 'Perfect, that works') that the pre-fix regex used to match -- a real regression for session.guided_mode=True sessions (which never reach the LLM-first gateway fallback). Fixed: loosened to ^(?:great|perfect)\b[\s,!.]*(?:let'?s?\s+go|that'?s?\s+(?:works|good|right))?$ -- restores the combined phrasings, keeps the original false-positive rejection intact. 2 pinning tests added in tests/test_cpq_post_approval_activation.py.</t>
         </is>
       </c>
       <c r="L44" s="4" t="inlineStr">

</xml_diff>